<commit_message>
update: nieuw invulformulier Rene (nu "René Charlataan") opnieuw uitgelezen
Oude voorspelling verwijderd, formulier opnieuw geparst en scorebord
herbouwd. Rene staat nu op positie 42 met 64 punten.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/formulieren/Invulformulier WK 2026 Rene.xlsx
+++ b/formulieren/Invulformulier WK 2026 Rene.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Thom\wk26-poule-wpcombogokspelsyndicaatbv\formulieren\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F5BA9E1-C2C6-4ED3-94D2-E9AC070F8A16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9B0E7A4-D2E8-482C-88B0-3BD43D8BCE56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -660,10 +660,10 @@
     <t>brazilië</t>
   </si>
   <si>
-    <t>Harry Kane</t>
-  </si>
-  <si>
-    <t>Rene</t>
+    <t>Vermalen</t>
+  </si>
+  <si>
+    <t>René Charlataan</t>
   </si>
 </sst>
 </file>
@@ -2322,7 +2322,7 @@
         <v>Zuid-Afrika</v>
       </c>
       <c r="H25" s="1">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I25" s="29" t="s">
         <v>23</v>
@@ -2359,13 +2359,13 @@
         <v>Paraguay</v>
       </c>
       <c r="H26" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I26" s="30" t="s">
         <v>23</v>
       </c>
       <c r="J26" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K26" s="10"/>
       <c r="L26" s="10"/>
@@ -2396,7 +2396,7 @@
         <v>Turkije</v>
       </c>
       <c r="H27" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I27" s="30" t="s">
         <v>23</v>
@@ -2433,13 +2433,13 @@
         <v>Japan</v>
       </c>
       <c r="H28" s="2">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I28" s="30" t="s">
         <v>23</v>
       </c>
       <c r="J28" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K28" s="10"/>
       <c r="L28" s="10"/>
@@ -2476,7 +2476,7 @@
         <v>23</v>
       </c>
       <c r="J29" s="4">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K29" s="10"/>
       <c r="L29" s="10"/>
@@ -2544,7 +2544,7 @@
         <v>Kroatië</v>
       </c>
       <c r="H31" s="2">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="I31" s="30" t="s">
         <v>23</v>
@@ -2581,13 +2581,13 @@
         <v>Zweden</v>
       </c>
       <c r="H32" s="2">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I32" s="30" t="s">
         <v>23</v>
       </c>
       <c r="J32" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K32" s="10"/>
       <c r="L32" s="10"/>
@@ -2618,13 +2618,13 @@
         <v>Iran</v>
       </c>
       <c r="H33" s="2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I33" s="30" t="s">
         <v>23</v>
       </c>
       <c r="J33" s="4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K33" s="10"/>
       <c r="L33" s="10"/>
@@ -2655,7 +2655,7 @@
         <v>Irak</v>
       </c>
       <c r="H34" s="2">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="I34" s="30" t="s">
         <v>23</v>
@@ -2692,13 +2692,13 @@
         <v>Nederland</v>
       </c>
       <c r="H35" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I35" s="30" t="s">
         <v>23</v>
       </c>
       <c r="J35" s="4">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K35" s="10"/>
       <c r="L35" s="10"/>
@@ -2735,7 +2735,7 @@
         <v>23</v>
       </c>
       <c r="J36" s="4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K36" s="10"/>
       <c r="L36" s="10"/>
@@ -2766,13 +2766,13 @@
         <v>Portugal</v>
       </c>
       <c r="H37" s="2">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I37" s="30" t="s">
         <v>23</v>
       </c>
       <c r="J37" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K37" s="10"/>
       <c r="L37" s="10"/>
@@ -2873,14 +2873,14 @@
       </c>
       <c r="C41" s="61"/>
       <c r="D41" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E41" s="36" t="str">
         <f>E6</f>
         <v>Canada</v>
       </c>
       <c r="F41" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G41" s="36" t="str">
         <f>G6</f>
@@ -2921,14 +2921,14 @@
         <v>Bosnië-Herzegovina</v>
       </c>
       <c r="F42" s="7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G42" s="36" t="str">
         <f t="shared" ref="G42:G44" si="2">G7</f>
         <v>Marokko</v>
       </c>
       <c r="H42" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I42" s="57" t="str">
         <f t="shared" ref="I42:I44" si="3">I7</f>
@@ -2937,7 +2937,7 @@
       <c r="J42" s="57"/>
       <c r="K42" s="57"/>
       <c r="L42" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M42" s="9"/>
       <c r="N42" s="21" t="s">
@@ -2955,14 +2955,14 @@
       </c>
       <c r="C43" s="57"/>
       <c r="D43" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E43" s="36" t="str">
         <f t="shared" si="1"/>
         <v>Qatar</v>
       </c>
       <c r="F43" s="7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G43" s="36" t="str">
         <f t="shared" si="2"/>
@@ -3010,7 +3010,7 @@
         <v>Schotland</v>
       </c>
       <c r="H44" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I44" s="57" t="str">
         <f t="shared" si="3"/>
@@ -3019,7 +3019,7 @@
       <c r="J44" s="57"/>
       <c r="K44" s="57"/>
       <c r="L44" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M44" s="9"/>
       <c r="N44" s="21" t="s">
@@ -3102,7 +3102,7 @@
         <v>Nederland</v>
       </c>
       <c r="F47" s="6">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G47" s="36" t="str">
         <f>G12</f>
@@ -3143,7 +3143,7 @@
         <v>Japan</v>
       </c>
       <c r="F48" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G48" s="36" t="str">
         <f t="shared" ref="G48:G50" si="6">G13</f>
@@ -3177,21 +3177,21 @@
       </c>
       <c r="C49" s="57"/>
       <c r="D49" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E49" s="36" t="str">
         <f t="shared" si="5"/>
         <v>Zweden</v>
       </c>
       <c r="F49" s="7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G49" s="36" t="str">
         <f t="shared" si="6"/>
         <v>Iran</v>
       </c>
       <c r="H49" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I49" s="57" t="str">
         <f t="shared" si="7"/>
@@ -3218,21 +3218,21 @@
       </c>
       <c r="C50" s="57"/>
       <c r="D50" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E50" s="36" t="str">
         <f t="shared" si="5"/>
         <v>Tunesië</v>
       </c>
       <c r="F50" s="7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G50" s="36" t="str">
         <f t="shared" si="6"/>
         <v>Nieuw-Zeeland</v>
       </c>
       <c r="H50" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I50" s="57" t="str">
         <f t="shared" si="7"/>
@@ -3340,7 +3340,7 @@
       <c r="J53" s="66"/>
       <c r="K53" s="67"/>
       <c r="L53" s="6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M53" s="9"/>
       <c r="N53" s="9"/>
@@ -3354,21 +3354,21 @@
       </c>
       <c r="C54" s="57"/>
       <c r="D54" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E54" s="36" t="str">
         <f t="shared" ref="E54:E56" si="9">E19</f>
         <v>Algerije</v>
       </c>
       <c r="F54" s="7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G54" s="36" t="str">
         <f t="shared" ref="G54:G56" si="10">G19</f>
         <v>DR Congo</v>
       </c>
       <c r="H54" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I54" s="57" t="str">
         <f t="shared" ref="I54:I56" si="11">I19</f>
@@ -3377,7 +3377,7 @@
       <c r="J54" s="57"/>
       <c r="K54" s="57"/>
       <c r="L54" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M54" s="9"/>
       <c r="N54" s="9"/>
@@ -3398,14 +3398,14 @@
         <v>Oostenrijk</v>
       </c>
       <c r="F55" s="7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G55" s="36" t="str">
         <f t="shared" si="10"/>
         <v>Oezbekistan</v>
       </c>
       <c r="H55" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I55" s="57" t="str">
         <f t="shared" si="11"/>
@@ -3414,7 +3414,7 @@
       <c r="J55" s="57"/>
       <c r="K55" s="57"/>
       <c r="L55" s="4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M55" s="9"/>
       <c r="N55" s="9"/>
@@ -3428,7 +3428,7 @@
       </c>
       <c r="C56" s="57"/>
       <c r="D56" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E56" s="36" t="str">
         <f t="shared" si="9"/>
@@ -3442,7 +3442,7 @@
         <v>Colombia</v>
       </c>
       <c r="H56" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I56" s="57" t="str">
         <f t="shared" si="11"/>
@@ -3451,7 +3451,7 @@
       <c r="J56" s="57"/>
       <c r="K56" s="57"/>
       <c r="L56" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M56" s="9"/>
       <c r="N56" s="9"/>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="G60" s="47"/>
       <c r="H60" s="53" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="I60" s="53"/>
       <c r="J60" s="53"/>
@@ -3626,7 +3626,7 @@
       </c>
       <c r="G63" s="48"/>
       <c r="H63" s="49" t="s">
-        <v>180</v>
+        <v>87</v>
       </c>
       <c r="I63" s="49"/>
       <c r="J63" s="49"/>
@@ -3688,7 +3688,7 @@
       </c>
       <c r="G65" s="48"/>
       <c r="H65" s="49" t="s">
-        <v>183</v>
+        <v>14</v>
       </c>
       <c r="I65" s="49"/>
       <c r="J65" s="49"/>
@@ -3719,7 +3719,7 @@
       </c>
       <c r="G66" s="48"/>
       <c r="H66" s="49" t="s">
-        <v>203</v>
+        <v>20</v>
       </c>
       <c r="I66" s="49"/>
       <c r="J66" s="49"/>
@@ -3750,7 +3750,7 @@
       </c>
       <c r="G67" s="48"/>
       <c r="H67" s="49" t="s">
-        <v>186</v>
+        <v>9</v>
       </c>
       <c r="I67" s="49"/>
       <c r="J67" s="49"/>
@@ -3781,7 +3781,7 @@
       </c>
       <c r="G68" s="47"/>
       <c r="H68" s="53" t="s">
-        <v>188</v>
+        <v>17</v>
       </c>
       <c r="I68" s="53"/>
       <c r="J68" s="53"/>
@@ -3812,7 +3812,7 @@
       </c>
       <c r="G69" s="48"/>
       <c r="H69" s="49" t="s">
-        <v>190</v>
+        <v>82</v>
       </c>
       <c r="I69" s="49"/>
       <c r="J69" s="49"/>
@@ -3843,7 +3843,7 @@
       </c>
       <c r="G70" s="48"/>
       <c r="H70" s="49" t="s">
-        <v>192</v>
+        <v>7</v>
       </c>
       <c r="I70" s="49"/>
       <c r="J70" s="49"/>
@@ -3874,7 +3874,7 @@
       </c>
       <c r="G71" s="48"/>
       <c r="H71" s="49" t="s">
-        <v>204</v>
+        <v>13</v>
       </c>
       <c r="I71" s="49"/>
       <c r="J71" s="49"/>
@@ -3905,7 +3905,7 @@
       </c>
       <c r="G72" s="48"/>
       <c r="H72" s="49" t="s">
-        <v>196</v>
+        <v>12</v>
       </c>
       <c r="I72" s="49"/>
       <c r="J72" s="49"/>
@@ -3936,7 +3936,7 @@
       </c>
       <c r="G73" s="48"/>
       <c r="H73" s="49" t="s">
-        <v>197</v>
+        <v>18</v>
       </c>
       <c r="I73" s="49"/>
       <c r="J73" s="49"/>
@@ -3967,7 +3967,7 @@
       </c>
       <c r="G74" s="48"/>
       <c r="H74" s="49" t="s">
-        <v>201</v>
+        <v>99</v>
       </c>
       <c r="I74" s="49"/>
       <c r="J74" s="49"/>
@@ -3998,7 +3998,7 @@
       </c>
       <c r="G75" s="48"/>
       <c r="H75" s="49" t="s">
-        <v>199</v>
+        <v>19</v>
       </c>
       <c r="I75" s="49"/>
       <c r="J75" s="49"/>
@@ -4084,7 +4084,7 @@
       </c>
       <c r="G79" s="47"/>
       <c r="H79" s="53" t="s">
-        <v>180</v>
+        <v>87</v>
       </c>
       <c r="I79" s="53"/>
       <c r="J79" s="53"/>
@@ -4115,7 +4115,7 @@
       </c>
       <c r="G80" s="48"/>
       <c r="H80" s="49" t="s">
-        <v>178</v>
+        <v>14</v>
       </c>
       <c r="I80" s="49"/>
       <c r="J80" s="49"/>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="G81" s="48"/>
       <c r="H81" s="49" t="s">
-        <v>206</v>
+        <v>78</v>
       </c>
       <c r="I81" s="49"/>
       <c r="J81" s="49"/>
@@ -4177,7 +4177,7 @@
       </c>
       <c r="G82" s="48"/>
       <c r="H82" s="49" t="s">
-        <v>186</v>
+        <v>9</v>
       </c>
       <c r="I82" s="49"/>
       <c r="J82" s="49"/>
@@ -4208,7 +4208,7 @@
       </c>
       <c r="G83" s="48"/>
       <c r="H83" s="49" t="s">
-        <v>192</v>
+        <v>13</v>
       </c>
       <c r="I83" s="49"/>
       <c r="J83" s="49"/>
@@ -4239,7 +4239,7 @@
       </c>
       <c r="G84" s="48"/>
       <c r="H84" s="49" t="s">
-        <v>188</v>
+        <v>82</v>
       </c>
       <c r="I84" s="49"/>
       <c r="J84" s="49"/>
@@ -4270,7 +4270,7 @@
       </c>
       <c r="G85" s="48"/>
       <c r="H85" s="49" t="s">
-        <v>201</v>
+        <v>99</v>
       </c>
       <c r="I85" s="49"/>
       <c r="J85" s="49"/>
@@ -4301,7 +4301,7 @@
       </c>
       <c r="G86" s="48"/>
       <c r="H86" s="49" t="s">
-        <v>199</v>
+        <v>19</v>
       </c>
       <c r="I86" s="49"/>
       <c r="J86" s="49"/>
@@ -4383,7 +4383,7 @@
       </c>
       <c r="G90" s="48"/>
       <c r="H90" s="53" t="s">
-        <v>180</v>
+        <v>14</v>
       </c>
       <c r="I90" s="53"/>
       <c r="J90" s="53"/>
@@ -4410,7 +4410,7 @@
       </c>
       <c r="G91" s="48"/>
       <c r="H91" s="49" t="s">
-        <v>192</v>
+        <v>13</v>
       </c>
       <c r="I91" s="49"/>
       <c r="J91" s="49"/>
@@ -4437,7 +4437,7 @@
       </c>
       <c r="G92" s="48"/>
       <c r="H92" s="49" t="s">
-        <v>186</v>
+        <v>9</v>
       </c>
       <c r="I92" s="49"/>
       <c r="J92" s="49"/>
@@ -4464,7 +4464,7 @@
       </c>
       <c r="G93" s="48"/>
       <c r="H93" s="49" t="s">
-        <v>199</v>
+        <v>19</v>
       </c>
       <c r="I93" s="49"/>
       <c r="J93" s="49"/>
@@ -4546,7 +4546,7 @@
       </c>
       <c r="G97" s="48"/>
       <c r="H97" s="53" t="s">
-        <v>180</v>
+        <v>14</v>
       </c>
       <c r="I97" s="53"/>
       <c r="J97" s="53"/>
@@ -4573,7 +4573,7 @@
       </c>
       <c r="G98" s="48"/>
       <c r="H98" s="49" t="s">
-        <v>186</v>
+        <v>19</v>
       </c>
       <c r="I98" s="49"/>
       <c r="J98" s="49"/>
@@ -4634,7 +4634,7 @@
         <v>57</v>
       </c>
       <c r="H101" s="53" t="s">
-        <v>186</v>
+        <v>14</v>
       </c>
       <c r="I101" s="53"/>
       <c r="J101" s="53"/>
@@ -4655,7 +4655,7 @@
         <v>58</v>
       </c>
       <c r="H102" s="49" t="s">
-        <v>180</v>
+        <v>19</v>
       </c>
       <c r="I102" s="49"/>
       <c r="J102" s="49"/>
@@ -4693,7 +4693,7 @@
       <c r="D104" s="48"/>
       <c r="E104" s="48"/>
       <c r="F104" s="5">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="G104" s="9"/>
       <c r="H104" s="9"/>
@@ -4714,7 +4714,7 @@
       <c r="D105" s="48"/>
       <c r="E105" s="48"/>
       <c r="F105" s="5">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G105" s="9"/>
       <c r="H105" s="9"/>
@@ -4735,7 +4735,7 @@
       <c r="D106" s="48"/>
       <c r="E106" s="48"/>
       <c r="F106" s="5">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="G106" s="9"/>
       <c r="H106" s="9"/>
@@ -4756,7 +4756,7 @@
       <c r="D107" s="48"/>
       <c r="E107" s="48"/>
       <c r="F107" s="5">
-        <v>278</v>
+        <v>291</v>
       </c>
       <c r="G107" s="72"/>
       <c r="H107" s="73"/>
@@ -4777,7 +4777,7 @@
       <c r="D108" s="48"/>
       <c r="E108" s="48"/>
       <c r="F108" s="5">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="G108" s="72"/>
       <c r="H108" s="73"/>

</xml_diff>

<commit_message>
Grap-onthulling René: handicap eraf en topscorer gecorrigeerd
De +50-handicap vervalt nu direct (niet meer wachtend op de finale) en de
naam wordt onthuld als "René 'zonder +50' Aan" — sommigen namen het te
serieus. Topscorer 'Vermalen' in het formulier gecorrigeerd naar Donyell Malen.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/formulieren/Invulformulier WK 2026 Rene.xlsx
+++ b/formulieren/Invulformulier WK 2026 Rene.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Thom\wk26-poule-wpcombogokspelsyndicaatbv\formulieren\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9B0E7A4-D2E8-482C-88B0-3BD43D8BCE56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A4012C8-3EFF-4DD6-8875-43F385E93FC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5220" yWindow="3165" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="invulformulier" sheetId="81" r:id="rId1"/>
@@ -660,10 +660,10 @@
     <t>brazilië</t>
   </si>
   <si>
-    <t>Vermalen</t>
-  </si>
-  <si>
     <t>René Charlataan</t>
+  </si>
+  <si>
+    <t>Donyell Malen</t>
   </si>
 </sst>
 </file>
@@ -1203,32 +1203,71 @@
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1237,18 +1276,18 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="24" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1256,51 +1295,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="25" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1640,9 +1640,9 @@
       <c r="F1" s="9"/>
       <c r="G1" s="9"/>
       <c r="H1" s="9"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
+      <c r="I1" s="60"/>
+      <c r="J1" s="60"/>
+      <c r="K1" s="60"/>
       <c r="L1" s="10"/>
       <c r="M1" s="10"/>
       <c r="N1" s="10"/>
@@ -1650,23 +1650,23 @@
     </row>
     <row r="2" spans="1:15" s="15" customFormat="1" ht="20.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="9"/>
-      <c r="B2" s="78" t="s">
+      <c r="B2" s="65" t="s">
         <v>175</v>
       </c>
-      <c r="C2" s="79"/>
-      <c r="D2" s="79"/>
-      <c r="E2" s="80"/>
+      <c r="C2" s="66"/>
+      <c r="D2" s="66"/>
+      <c r="E2" s="67"/>
       <c r="F2" s="9"/>
       <c r="G2" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="H2" s="75" t="s">
-        <v>208</v>
-      </c>
-      <c r="I2" s="76"/>
-      <c r="J2" s="76"/>
-      <c r="K2" s="76"/>
-      <c r="L2" s="77"/>
+      <c r="H2" s="62" t="s">
+        <v>207</v>
+      </c>
+      <c r="I2" s="63"/>
+      <c r="J2" s="63"/>
+      <c r="K2" s="63"/>
+      <c r="L2" s="64"/>
       <c r="M2" s="13"/>
       <c r="N2" s="14"/>
       <c r="O2" s="11"/>
@@ -1690,19 +1690,19 @@
     </row>
     <row r="4" spans="1:15" s="15" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9"/>
-      <c r="B4" s="74" t="s">
+      <c r="B4" s="61" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="74"/>
-      <c r="D4" s="74"/>
-      <c r="E4" s="74"/>
-      <c r="F4" s="74"/>
-      <c r="G4" s="74"/>
-      <c r="H4" s="74"/>
-      <c r="I4" s="74"/>
-      <c r="J4" s="74"/>
-      <c r="K4" s="74"/>
-      <c r="L4" s="74"/>
+      <c r="C4" s="61"/>
+      <c r="D4" s="61"/>
+      <c r="E4" s="61"/>
+      <c r="F4" s="61"/>
+      <c r="G4" s="61"/>
+      <c r="H4" s="61"/>
+      <c r="I4" s="61"/>
+      <c r="J4" s="61"/>
+      <c r="K4" s="61"/>
+      <c r="L4" s="61"/>
       <c r="M4" s="11"/>
       <c r="N4" s="16" t="s">
         <v>107</v>
@@ -1713,25 +1713,25 @@
     </row>
     <row r="5" spans="1:15" s="15" customFormat="1" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A5" s="9"/>
-      <c r="B5" s="71" t="s">
+      <c r="B5" s="57" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="71"/>
-      <c r="D5" s="71"/>
-      <c r="E5" s="71" t="s">
+      <c r="C5" s="57"/>
+      <c r="D5" s="57"/>
+      <c r="E5" s="57" t="s">
         <v>3</v>
       </c>
-      <c r="F5" s="71"/>
-      <c r="G5" s="71" t="s">
+      <c r="F5" s="57"/>
+      <c r="G5" s="57" t="s">
         <v>4</v>
       </c>
-      <c r="H5" s="71"/>
-      <c r="I5" s="71" t="s">
+      <c r="H5" s="57"/>
+      <c r="I5" s="57" t="s">
         <v>5</v>
       </c>
-      <c r="J5" s="71"/>
-      <c r="K5" s="71"/>
-      <c r="L5" s="71"/>
+      <c r="J5" s="57"/>
+      <c r="K5" s="57"/>
+      <c r="L5" s="57"/>
       <c r="M5" s="17"/>
       <c r="N5" s="18" t="s">
         <v>72</v>
@@ -1742,11 +1742,11 @@
     </row>
     <row r="6" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A6" s="9"/>
-      <c r="B6" s="58" t="str">
+      <c r="B6" s="50" t="str">
         <f>N5</f>
         <v>Mexico</v>
       </c>
-      <c r="C6" s="81"/>
+      <c r="C6" s="68"/>
       <c r="D6" s="47"/>
       <c r="E6" s="48" t="str">
         <f>N9</f>
@@ -1775,11 +1775,11 @@
     </row>
     <row r="7" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A7" s="9"/>
-      <c r="B7" s="58" t="str">
+      <c r="B7" s="50" t="str">
         <f>N6</f>
         <v>Zuid-Afrika</v>
       </c>
-      <c r="C7" s="81"/>
+      <c r="C7" s="68"/>
       <c r="D7" s="47"/>
       <c r="E7" s="48" t="str">
         <f>N10</f>
@@ -1808,11 +1808,11 @@
     </row>
     <row r="8" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A8" s="9"/>
-      <c r="B8" s="58" t="str">
+      <c r="B8" s="50" t="str">
         <f>N7</f>
         <v>Zuid-Korea</v>
       </c>
-      <c r="C8" s="81"/>
+      <c r="C8" s="68"/>
       <c r="D8" s="47"/>
       <c r="E8" s="48" t="str">
         <f>N11</f>
@@ -1841,12 +1841,12 @@
     </row>
     <row r="9" spans="1:15" s="15" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="9"/>
-      <c r="B9" s="50" t="str">
+      <c r="B9" s="54" t="str">
         <f>N8</f>
         <v>Tsjechië</v>
       </c>
-      <c r="C9" s="51"/>
-      <c r="D9" s="52"/>
+      <c r="C9" s="55"/>
+      <c r="D9" s="56"/>
       <c r="E9" s="48" t="str">
         <f>N12</f>
         <v>Zwitserland</v>
@@ -1874,17 +1874,17 @@
     </row>
     <row r="10" spans="1:15" s="15" customFormat="1" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="9"/>
-      <c r="B10" s="70"/>
-      <c r="C10" s="70"/>
-      <c r="D10" s="70"/>
-      <c r="E10" s="70"/>
-      <c r="F10" s="70"/>
-      <c r="G10" s="70"/>
-      <c r="H10" s="70"/>
-      <c r="I10" s="70"/>
-      <c r="J10" s="70"/>
-      <c r="K10" s="70"/>
-      <c r="L10" s="70"/>
+      <c r="B10" s="80"/>
+      <c r="C10" s="80"/>
+      <c r="D10" s="80"/>
+      <c r="E10" s="80"/>
+      <c r="F10" s="80"/>
+      <c r="G10" s="80"/>
+      <c r="H10" s="80"/>
+      <c r="I10" s="80"/>
+      <c r="J10" s="80"/>
+      <c r="K10" s="80"/>
+      <c r="L10" s="80"/>
       <c r="M10" s="11"/>
       <c r="N10" s="21" t="s">
         <v>76</v>
@@ -1895,25 +1895,25 @@
     </row>
     <row r="11" spans="1:15" s="15" customFormat="1" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A11" s="9"/>
-      <c r="B11" s="71" t="s">
+      <c r="B11" s="57" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="71"/>
-      <c r="D11" s="71"/>
-      <c r="E11" s="71" t="s">
+      <c r="C11" s="57"/>
+      <c r="D11" s="57"/>
+      <c r="E11" s="57" t="s">
         <v>16</v>
       </c>
-      <c r="F11" s="71"/>
-      <c r="G11" s="71" t="s">
+      <c r="F11" s="57"/>
+      <c r="G11" s="57" t="s">
         <v>66</v>
       </c>
-      <c r="H11" s="71"/>
-      <c r="I11" s="71" t="s">
+      <c r="H11" s="57"/>
+      <c r="I11" s="57" t="s">
         <v>67</v>
       </c>
-      <c r="J11" s="71"/>
-      <c r="K11" s="71"/>
-      <c r="L11" s="71"/>
+      <c r="J11" s="57"/>
+      <c r="K11" s="57"/>
+      <c r="L11" s="57"/>
       <c r="M11" s="11"/>
       <c r="N11" s="21" t="s">
         <v>77</v>
@@ -2077,25 +2077,25 @@
     </row>
     <row r="17" spans="1:15" s="15" customFormat="1" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A17" s="9"/>
-      <c r="B17" s="71" t="s">
+      <c r="B17" s="57" t="s">
         <v>68</v>
       </c>
-      <c r="C17" s="71"/>
-      <c r="D17" s="71"/>
-      <c r="E17" s="71" t="s">
+      <c r="C17" s="57"/>
+      <c r="D17" s="57"/>
+      <c r="E17" s="57" t="s">
         <v>69</v>
       </c>
-      <c r="F17" s="71"/>
-      <c r="G17" s="71" t="s">
+      <c r="F17" s="57"/>
+      <c r="G17" s="57" t="s">
         <v>70</v>
       </c>
-      <c r="H17" s="71"/>
-      <c r="I17" s="71" t="s">
+      <c r="H17" s="57"/>
+      <c r="I17" s="57" t="s">
         <v>71</v>
       </c>
-      <c r="J17" s="71"/>
-      <c r="K17" s="71"/>
-      <c r="L17" s="71"/>
+      <c r="J17" s="57"/>
+      <c r="K17" s="57"/>
+      <c r="L17" s="57"/>
       <c r="M17" s="10"/>
       <c r="N17" s="21" t="s">
         <v>81</v>
@@ -2288,11 +2288,11 @@
       <c r="E24" s="9"/>
       <c r="F24" s="9"/>
       <c r="G24" s="9"/>
-      <c r="H24" s="62" t="s">
+      <c r="H24" s="73" t="s">
         <v>22</v>
       </c>
-      <c r="I24" s="63"/>
-      <c r="J24" s="64"/>
+      <c r="I24" s="74"/>
+      <c r="J24" s="75"/>
       <c r="K24" s="10"/>
       <c r="L24" s="10"/>
       <c r="M24" s="10"/>
@@ -2305,10 +2305,10 @@
     </row>
     <row r="25" spans="1:15" s="15" customFormat="1" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A25" s="9"/>
-      <c r="B25" s="68">
+      <c r="B25" s="69">
         <v>46184</v>
       </c>
-      <c r="C25" s="69"/>
+      <c r="C25" s="70"/>
       <c r="D25" s="25"/>
       <c r="E25" s="26" t="str">
         <f>B6</f>
@@ -2342,10 +2342,10 @@
     </row>
     <row r="26" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A26" s="9"/>
-      <c r="B26" s="68">
+      <c r="B26" s="69">
         <v>46185</v>
       </c>
-      <c r="C26" s="69"/>
+      <c r="C26" s="70"/>
       <c r="D26" s="25"/>
       <c r="E26" s="26" t="str">
         <f>I6</f>
@@ -2379,10 +2379,10 @@
     </row>
     <row r="27" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A27" s="9"/>
-      <c r="B27" s="68">
+      <c r="B27" s="69">
         <v>46186</v>
       </c>
-      <c r="C27" s="69"/>
+      <c r="C27" s="70"/>
       <c r="D27" s="25"/>
       <c r="E27" s="26" t="str">
         <f>I8</f>
@@ -2416,10 +2416,10 @@
     </row>
     <row r="28" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A28" s="9"/>
-      <c r="B28" s="68">
+      <c r="B28" s="69">
         <v>46187</v>
       </c>
-      <c r="C28" s="69"/>
+      <c r="C28" s="70"/>
       <c r="D28" s="25"/>
       <c r="E28" s="26" t="str">
         <f>E12</f>
@@ -2453,10 +2453,10 @@
     </row>
     <row r="29" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A29" s="9"/>
-      <c r="B29" s="68">
+      <c r="B29" s="69">
         <v>46187</v>
       </c>
-      <c r="C29" s="69"/>
+      <c r="C29" s="70"/>
       <c r="D29" s="25"/>
       <c r="E29" s="33" t="str">
         <f>B12</f>
@@ -2490,10 +2490,10 @@
     </row>
     <row r="30" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A30" s="9"/>
-      <c r="B30" s="68">
+      <c r="B30" s="69">
         <v>46189</v>
       </c>
-      <c r="C30" s="69"/>
+      <c r="C30" s="70"/>
       <c r="D30" s="25"/>
       <c r="E30" s="33" t="str">
         <f>E18</f>
@@ -2527,10 +2527,10 @@
     </row>
     <row r="31" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A31" s="9"/>
-      <c r="B31" s="68">
+      <c r="B31" s="69">
         <v>46190</v>
       </c>
-      <c r="C31" s="69"/>
+      <c r="C31" s="70"/>
       <c r="D31" s="25"/>
       <c r="E31" s="33" t="str">
         <f>I18</f>
@@ -2564,10 +2564,10 @@
     </row>
     <row r="32" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A32" s="9"/>
-      <c r="B32" s="68">
+      <c r="B32" s="69">
         <v>46193</v>
       </c>
-      <c r="C32" s="69"/>
+      <c r="C32" s="70"/>
       <c r="D32" s="25"/>
       <c r="E32" s="33" t="str">
         <f>E12</f>
@@ -2601,10 +2601,10 @@
     </row>
     <row r="33" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A33" s="9"/>
-      <c r="B33" s="68">
+      <c r="B33" s="69">
         <v>46194</v>
       </c>
-      <c r="C33" s="69"/>
+      <c r="C33" s="70"/>
       <c r="D33" s="25"/>
       <c r="E33" s="33" t="str">
         <f>G12</f>
@@ -2638,10 +2638,10 @@
     </row>
     <row r="34" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A34" s="9"/>
-      <c r="B34" s="68">
+      <c r="B34" s="69">
         <v>46195</v>
       </c>
-      <c r="C34" s="69"/>
+      <c r="C34" s="70"/>
       <c r="D34" s="25"/>
       <c r="E34" s="33" t="str">
         <f>B18</f>
@@ -2675,10 +2675,10 @@
     </row>
     <row r="35" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A35" s="9"/>
-      <c r="B35" s="68">
+      <c r="B35" s="69">
         <v>46198</v>
       </c>
-      <c r="C35" s="69"/>
+      <c r="C35" s="70"/>
       <c r="D35" s="25"/>
       <c r="E35" s="33" t="str">
         <f>E15</f>
@@ -2712,10 +2712,10 @@
     </row>
     <row r="36" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A36" s="9"/>
-      <c r="B36" s="68">
+      <c r="B36" s="69">
         <v>46198</v>
       </c>
-      <c r="C36" s="69"/>
+      <c r="C36" s="70"/>
       <c r="D36" s="25"/>
       <c r="E36" s="33" t="str">
         <f>B13</f>
@@ -2749,10 +2749,10 @@
     </row>
     <row r="37" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A37" s="9"/>
-      <c r="B37" s="68">
+      <c r="B37" s="69">
         <v>46200</v>
       </c>
-      <c r="C37" s="69"/>
+      <c r="C37" s="70"/>
       <c r="D37" s="25"/>
       <c r="E37" s="33" t="str">
         <f>G21</f>
@@ -2807,20 +2807,20 @@
     </row>
     <row r="39" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A39" s="9"/>
-      <c r="B39" s="56" t="s">
+      <c r="B39" s="53" t="s">
         <v>24</v>
       </c>
-      <c r="C39" s="56"/>
-      <c r="D39" s="56"/>
-      <c r="E39" s="56"/>
-      <c r="F39" s="56"/>
-      <c r="G39" s="56"/>
-      <c r="H39" s="56"/>
-      <c r="I39" s="56"/>
-      <c r="J39" s="56"/>
-      <c r="K39" s="56"/>
-      <c r="L39" s="56"/>
-      <c r="M39" s="56"/>
+      <c r="C39" s="53"/>
+      <c r="D39" s="53"/>
+      <c r="E39" s="53"/>
+      <c r="F39" s="53"/>
+      <c r="G39" s="53"/>
+      <c r="H39" s="53"/>
+      <c r="I39" s="53"/>
+      <c r="J39" s="53"/>
+      <c r="K39" s="53"/>
+      <c r="L39" s="53"/>
+      <c r="M39" s="53"/>
       <c r="N39" s="21" t="s">
         <v>97</v>
       </c>
@@ -2830,10 +2830,10 @@
     </row>
     <row r="40" spans="1:15" s="15" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="9"/>
-      <c r="B40" s="59" t="s">
+      <c r="B40" s="71" t="s">
         <v>2</v>
       </c>
-      <c r="C40" s="60"/>
+      <c r="C40" s="72"/>
       <c r="D40" s="35" t="s">
         <v>25</v>
       </c>
@@ -2849,11 +2849,11 @@
       <c r="H40" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="I40" s="62" t="s">
+      <c r="I40" s="73" t="s">
         <v>5</v>
       </c>
-      <c r="J40" s="63"/>
-      <c r="K40" s="64"/>
+      <c r="J40" s="74"/>
+      <c r="K40" s="75"/>
       <c r="L40" s="35" t="s">
         <v>25</v>
       </c>
@@ -2867,11 +2867,11 @@
     </row>
     <row r="41" spans="1:15" s="15" customFormat="1" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A41" s="9"/>
-      <c r="B41" s="61" t="str">
+      <c r="B41" s="76" t="str">
         <f>B6</f>
         <v>Mexico</v>
       </c>
-      <c r="C41" s="61"/>
+      <c r="C41" s="76"/>
       <c r="D41" s="3">
         <v>2</v>
       </c>
@@ -2889,12 +2889,12 @@
       <c r="H41" s="6">
         <v>1</v>
       </c>
-      <c r="I41" s="65" t="str">
+      <c r="I41" s="77" t="str">
         <f>I6</f>
         <v>Verenigde Staten</v>
       </c>
-      <c r="J41" s="66"/>
-      <c r="K41" s="67"/>
+      <c r="J41" s="78"/>
+      <c r="K41" s="79"/>
       <c r="L41" s="6">
         <v>3</v>
       </c>
@@ -2908,11 +2908,11 @@
     </row>
     <row r="42" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A42" s="9"/>
-      <c r="B42" s="57" t="str">
+      <c r="B42" s="52" t="str">
         <f t="shared" ref="B42:B44" si="0">B7</f>
         <v>Zuid-Afrika</v>
       </c>
-      <c r="C42" s="57"/>
+      <c r="C42" s="52"/>
       <c r="D42" s="4">
         <v>4</v>
       </c>
@@ -2930,12 +2930,12 @@
       <c r="H42" s="2">
         <v>3</v>
       </c>
-      <c r="I42" s="57" t="str">
+      <c r="I42" s="52" t="str">
         <f t="shared" ref="I42:I44" si="3">I7</f>
         <v>Paraguay</v>
       </c>
-      <c r="J42" s="57"/>
-      <c r="K42" s="57"/>
+      <c r="J42" s="52"/>
+      <c r="K42" s="52"/>
       <c r="L42" s="4">
         <v>1</v>
       </c>
@@ -2949,11 +2949,11 @@
     </row>
     <row r="43" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A43" s="9"/>
-      <c r="B43" s="57" t="str">
+      <c r="B43" s="52" t="str">
         <f t="shared" si="0"/>
         <v>Zuid-Korea</v>
       </c>
-      <c r="C43" s="57"/>
+      <c r="C43" s="52"/>
       <c r="D43" s="4">
         <v>3</v>
       </c>
@@ -2971,12 +2971,12 @@
       <c r="H43" s="2">
         <v>4</v>
       </c>
-      <c r="I43" s="57" t="str">
+      <c r="I43" s="52" t="str">
         <f t="shared" si="3"/>
         <v>Australië</v>
       </c>
-      <c r="J43" s="57"/>
-      <c r="K43" s="57"/>
+      <c r="J43" s="52"/>
+      <c r="K43" s="52"/>
       <c r="L43" s="4">
         <v>4</v>
       </c>
@@ -2990,11 +2990,11 @@
     </row>
     <row r="44" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A44" s="9"/>
-      <c r="B44" s="57" t="str">
+      <c r="B44" s="52" t="str">
         <f t="shared" si="0"/>
         <v>Tsjechië</v>
       </c>
-      <c r="C44" s="57"/>
+      <c r="C44" s="52"/>
       <c r="D44" s="4">
         <v>1</v>
       </c>
@@ -3012,12 +3012,12 @@
       <c r="H44" s="2">
         <v>2</v>
       </c>
-      <c r="I44" s="57" t="str">
+      <c r="I44" s="52" t="str">
         <f t="shared" si="3"/>
         <v>Turkije</v>
       </c>
-      <c r="J44" s="57"/>
-      <c r="K44" s="57"/>
+      <c r="J44" s="52"/>
+      <c r="K44" s="52"/>
       <c r="L44" s="4">
         <v>2</v>
       </c>
@@ -3052,10 +3052,10 @@
     </row>
     <row r="46" spans="1:15" s="15" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A46" s="9"/>
-      <c r="B46" s="59" t="s">
+      <c r="B46" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="C46" s="60"/>
+      <c r="C46" s="72"/>
       <c r="D46" s="35" t="s">
         <v>25</v>
       </c>
@@ -3071,11 +3071,11 @@
       <c r="H46" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="I46" s="62" t="s">
+      <c r="I46" s="73" t="s">
         <v>67</v>
       </c>
-      <c r="J46" s="63"/>
-      <c r="K46" s="64"/>
+      <c r="J46" s="74"/>
+      <c r="K46" s="75"/>
       <c r="L46" s="35" t="s">
         <v>25</v>
       </c>
@@ -3089,11 +3089,11 @@
     </row>
     <row r="47" spans="1:15" s="15" customFormat="1" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A47" s="9"/>
-      <c r="B47" s="61" t="str">
+      <c r="B47" s="76" t="str">
         <f>B12</f>
         <v>Duitsland</v>
       </c>
-      <c r="C47" s="61"/>
+      <c r="C47" s="76"/>
       <c r="D47" s="3">
         <v>1</v>
       </c>
@@ -3111,12 +3111,12 @@
       <c r="H47" s="6">
         <v>1</v>
       </c>
-      <c r="I47" s="65" t="str">
+      <c r="I47" s="77" t="str">
         <f>I12</f>
         <v>Spanje</v>
       </c>
-      <c r="J47" s="66"/>
-      <c r="K47" s="67"/>
+      <c r="J47" s="78"/>
+      <c r="K47" s="79"/>
       <c r="L47" s="6">
         <v>1</v>
       </c>
@@ -3130,11 +3130,11 @@
     </row>
     <row r="48" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A48" s="9"/>
-      <c r="B48" s="57" t="str">
+      <c r="B48" s="52" t="str">
         <f t="shared" ref="B48:B50" si="4">B13</f>
         <v>Curaçao</v>
       </c>
-      <c r="C48" s="57"/>
+      <c r="C48" s="52"/>
       <c r="D48" s="4">
         <v>2</v>
       </c>
@@ -3152,12 +3152,12 @@
       <c r="H48" s="2">
         <v>2</v>
       </c>
-      <c r="I48" s="57" t="str">
+      <c r="I48" s="52" t="str">
         <f t="shared" ref="I48:I50" si="7">I13</f>
         <v>Kaapverdië</v>
       </c>
-      <c r="J48" s="57"/>
-      <c r="K48" s="57"/>
+      <c r="J48" s="52"/>
+      <c r="K48" s="52"/>
       <c r="L48" s="4">
         <v>3</v>
       </c>
@@ -3171,11 +3171,11 @@
     </row>
     <row r="49" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A49" s="9"/>
-      <c r="B49" s="57" t="str">
+      <c r="B49" s="52" t="str">
         <f t="shared" si="4"/>
         <v>Ivoorkust</v>
       </c>
-      <c r="C49" s="57"/>
+      <c r="C49" s="52"/>
       <c r="D49" s="4">
         <v>4</v>
       </c>
@@ -3193,12 +3193,12 @@
       <c r="H49" s="2">
         <v>3</v>
       </c>
-      <c r="I49" s="57" t="str">
+      <c r="I49" s="52" t="str">
         <f t="shared" si="7"/>
         <v>Saoedi-Arabië</v>
       </c>
-      <c r="J49" s="57"/>
-      <c r="K49" s="57"/>
+      <c r="J49" s="52"/>
+      <c r="K49" s="52"/>
       <c r="L49" s="4">
         <v>4</v>
       </c>
@@ -3212,11 +3212,11 @@
     </row>
     <row r="50" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A50" s="9"/>
-      <c r="B50" s="57" t="str">
+      <c r="B50" s="52" t="str">
         <f t="shared" si="4"/>
         <v>Ecuador</v>
       </c>
-      <c r="C50" s="57"/>
+      <c r="C50" s="52"/>
       <c r="D50" s="4">
         <v>3</v>
       </c>
@@ -3234,12 +3234,12 @@
       <c r="H50" s="2">
         <v>4</v>
       </c>
-      <c r="I50" s="57" t="str">
+      <c r="I50" s="52" t="str">
         <f t="shared" si="7"/>
         <v>Uruguay</v>
       </c>
-      <c r="J50" s="57"/>
-      <c r="K50" s="57"/>
+      <c r="J50" s="52"/>
+      <c r="K50" s="52"/>
       <c r="L50" s="4">
         <v>2</v>
       </c>
@@ -3274,10 +3274,10 @@
     </row>
     <row r="52" spans="1:15" s="15" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="9"/>
-      <c r="B52" s="59" t="s">
+      <c r="B52" s="71" t="s">
         <v>68</v>
       </c>
-      <c r="C52" s="60"/>
+      <c r="C52" s="72"/>
       <c r="D52" s="35" t="s">
         <v>25</v>
       </c>
@@ -3293,11 +3293,11 @@
       <c r="H52" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="I52" s="62" t="s">
+      <c r="I52" s="73" t="s">
         <v>71</v>
       </c>
-      <c r="J52" s="63"/>
-      <c r="K52" s="64"/>
+      <c r="J52" s="74"/>
+      <c r="K52" s="75"/>
       <c r="L52" s="35" t="s">
         <v>25</v>
       </c>
@@ -3311,11 +3311,11 @@
     </row>
     <row r="53" spans="1:15" s="15" customFormat="1" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A53" s="9"/>
-      <c r="B53" s="61" t="str">
+      <c r="B53" s="76" t="str">
         <f>B18</f>
         <v>Frankrijk</v>
       </c>
-      <c r="C53" s="61"/>
+      <c r="C53" s="76"/>
       <c r="D53" s="3">
         <v>1</v>
       </c>
@@ -3333,12 +3333,12 @@
       <c r="H53" s="6">
         <v>1</v>
       </c>
-      <c r="I53" s="65" t="str">
+      <c r="I53" s="77" t="str">
         <f>I18</f>
         <v>Engeland</v>
       </c>
-      <c r="J53" s="66"/>
-      <c r="K53" s="67"/>
+      <c r="J53" s="78"/>
+      <c r="K53" s="79"/>
       <c r="L53" s="6">
         <v>2</v>
       </c>
@@ -3348,11 +3348,11 @@
     </row>
     <row r="54" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A54" s="9"/>
-      <c r="B54" s="57" t="str">
+      <c r="B54" s="52" t="str">
         <f t="shared" ref="B54:B56" si="8">B19</f>
         <v>Senegal</v>
       </c>
-      <c r="C54" s="57"/>
+      <c r="C54" s="52"/>
       <c r="D54" s="4">
         <v>3</v>
       </c>
@@ -3370,12 +3370,12 @@
       <c r="H54" s="2">
         <v>4</v>
       </c>
-      <c r="I54" s="57" t="str">
+      <c r="I54" s="52" t="str">
         <f t="shared" ref="I54:I56" si="11">I19</f>
         <v>Kroatië</v>
       </c>
-      <c r="J54" s="57"/>
-      <c r="K54" s="57"/>
+      <c r="J54" s="52"/>
+      <c r="K54" s="52"/>
       <c r="L54" s="4">
         <v>1</v>
       </c>
@@ -3385,11 +3385,11 @@
     </row>
     <row r="55" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A55" s="9"/>
-      <c r="B55" s="57" t="str">
+      <c r="B55" s="52" t="str">
         <f t="shared" si="8"/>
         <v>Irak</v>
       </c>
-      <c r="C55" s="57"/>
+      <c r="C55" s="52"/>
       <c r="D55" s="4">
         <v>4</v>
       </c>
@@ -3407,12 +3407,12 @@
       <c r="H55" s="2">
         <v>3</v>
       </c>
-      <c r="I55" s="57" t="str">
+      <c r="I55" s="52" t="str">
         <f t="shared" si="11"/>
         <v>Ghana</v>
       </c>
-      <c r="J55" s="57"/>
-      <c r="K55" s="57"/>
+      <c r="J55" s="52"/>
+      <c r="K55" s="52"/>
       <c r="L55" s="4">
         <v>4</v>
       </c>
@@ -3422,11 +3422,11 @@
     </row>
     <row r="56" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A56" s="9"/>
-      <c r="B56" s="57" t="str">
+      <c r="B56" s="52" t="str">
         <f t="shared" si="8"/>
         <v>Noorwegen</v>
       </c>
-      <c r="C56" s="57"/>
+      <c r="C56" s="52"/>
       <c r="D56" s="4">
         <v>2</v>
       </c>
@@ -3444,12 +3444,12 @@
       <c r="H56" s="2">
         <v>2</v>
       </c>
-      <c r="I56" s="57" t="str">
+      <c r="I56" s="52" t="str">
         <f t="shared" si="11"/>
         <v>Panama</v>
       </c>
-      <c r="J56" s="57"/>
-      <c r="K56" s="57"/>
+      <c r="J56" s="52"/>
+      <c r="K56" s="52"/>
       <c r="L56" s="4">
         <v>3</v>
       </c>
@@ -3476,20 +3476,20 @@
     </row>
     <row r="58" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A58" s="9"/>
-      <c r="B58" s="56" t="s">
+      <c r="B58" s="53" t="s">
         <v>109</v>
       </c>
-      <c r="C58" s="56"/>
-      <c r="D58" s="56"/>
-      <c r="E58" s="56"/>
-      <c r="F58" s="56"/>
-      <c r="G58" s="56"/>
-      <c r="H58" s="56"/>
-      <c r="I58" s="56"/>
-      <c r="J58" s="56"/>
-      <c r="K58" s="56"/>
-      <c r="L58" s="56"/>
-      <c r="M58" s="56"/>
+      <c r="C58" s="53"/>
+      <c r="D58" s="53"/>
+      <c r="E58" s="53"/>
+      <c r="F58" s="53"/>
+      <c r="G58" s="53"/>
+      <c r="H58" s="53"/>
+      <c r="I58" s="53"/>
+      <c r="J58" s="53"/>
+      <c r="K58" s="53"/>
+      <c r="L58" s="53"/>
+      <c r="M58" s="53"/>
       <c r="N58" s="9"/>
       <c r="O58" s="9"/>
     </row>
@@ -3501,11 +3501,11 @@
       <c r="E59" s="9"/>
       <c r="F59" s="9"/>
       <c r="G59" s="9"/>
-      <c r="H59" s="50" t="s">
+      <c r="H59" s="54" t="s">
         <v>27</v>
       </c>
-      <c r="I59" s="51"/>
-      <c r="J59" s="52"/>
+      <c r="I59" s="55"/>
+      <c r="J59" s="56"/>
       <c r="K59" s="9"/>
       <c r="L59" s="9"/>
       <c r="M59" s="9"/>
@@ -3528,15 +3528,15 @@
       <c r="E60" s="46" t="s">
         <v>176</v>
       </c>
-      <c r="F60" s="58" t="s">
+      <c r="F60" s="50" t="s">
         <v>30</v>
       </c>
       <c r="G60" s="47"/>
-      <c r="H60" s="53" t="s">
+      <c r="H60" s="51" t="s">
         <v>72</v>
       </c>
-      <c r="I60" s="53"/>
-      <c r="J60" s="53"/>
+      <c r="I60" s="51"/>
+      <c r="J60" s="51"/>
       <c r="K60" s="9"/>
       <c r="L60" s="9"/>
       <c r="M60" s="9"/>
@@ -3776,15 +3776,15 @@
       <c r="E68" s="46" t="s">
         <v>189</v>
       </c>
-      <c r="F68" s="58" t="s">
+      <c r="F68" s="50" t="s">
         <v>130</v>
       </c>
       <c r="G68" s="47"/>
-      <c r="H68" s="53" t="s">
+      <c r="H68" s="51" t="s">
         <v>17</v>
       </c>
-      <c r="I68" s="53"/>
-      <c r="J68" s="53"/>
+      <c r="I68" s="51"/>
+      <c r="J68" s="51"/>
       <c r="K68" s="9"/>
       <c r="L68" s="9"/>
       <c r="M68" s="9"/>
@@ -4027,20 +4027,20 @@
     </row>
     <row r="77" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A77" s="9"/>
-      <c r="B77" s="56" t="s">
+      <c r="B77" s="53" t="s">
         <v>26</v>
       </c>
-      <c r="C77" s="56"/>
-      <c r="D77" s="56"/>
-      <c r="E77" s="56"/>
-      <c r="F77" s="56"/>
-      <c r="G77" s="56"/>
-      <c r="H77" s="56"/>
-      <c r="I77" s="56"/>
-      <c r="J77" s="56"/>
-      <c r="K77" s="56"/>
-      <c r="L77" s="56"/>
-      <c r="M77" s="56"/>
+      <c r="C77" s="53"/>
+      <c r="D77" s="53"/>
+      <c r="E77" s="53"/>
+      <c r="F77" s="53"/>
+      <c r="G77" s="53"/>
+      <c r="H77" s="53"/>
+      <c r="I77" s="53"/>
+      <c r="J77" s="53"/>
+      <c r="K77" s="53"/>
+      <c r="L77" s="53"/>
+      <c r="M77" s="53"/>
       <c r="N77" s="9"/>
       <c r="O77" s="9"/>
     </row>
@@ -4052,11 +4052,11 @@
       <c r="E78" s="9"/>
       <c r="F78" s="9"/>
       <c r="G78" s="9"/>
-      <c r="H78" s="50" t="s">
+      <c r="H78" s="54" t="s">
         <v>27</v>
       </c>
-      <c r="I78" s="51"/>
-      <c r="J78" s="52"/>
+      <c r="I78" s="55"/>
+      <c r="J78" s="56"/>
       <c r="K78" s="9"/>
       <c r="L78" s="9"/>
       <c r="M78" s="9"/>
@@ -4079,15 +4079,15 @@
       <c r="E79" s="46" t="s">
         <v>180</v>
       </c>
-      <c r="F79" s="58" t="s">
+      <c r="F79" s="50" t="s">
         <v>149</v>
       </c>
       <c r="G79" s="47"/>
-      <c r="H79" s="53" t="s">
+      <c r="H79" s="51" t="s">
         <v>87</v>
       </c>
-      <c r="I79" s="53"/>
-      <c r="J79" s="53"/>
+      <c r="I79" s="51"/>
+      <c r="J79" s="51"/>
       <c r="K79" s="9"/>
       <c r="L79" s="9"/>
       <c r="M79" s="9"/>
@@ -4330,20 +4330,20 @@
     </row>
     <row r="88" spans="1:15" s="15" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A88" s="9"/>
-      <c r="B88" s="56" t="s">
+      <c r="B88" s="53" t="s">
         <v>48</v>
       </c>
-      <c r="C88" s="56"/>
-      <c r="D88" s="56"/>
-      <c r="E88" s="56"/>
-      <c r="F88" s="56"/>
-      <c r="G88" s="56"/>
-      <c r="H88" s="56"/>
-      <c r="I88" s="56"/>
-      <c r="J88" s="56"/>
-      <c r="K88" s="56"/>
-      <c r="L88" s="56"/>
-      <c r="M88" s="56"/>
+      <c r="C88" s="53"/>
+      <c r="D88" s="53"/>
+      <c r="E88" s="53"/>
+      <c r="F88" s="53"/>
+      <c r="G88" s="53"/>
+      <c r="H88" s="53"/>
+      <c r="I88" s="53"/>
+      <c r="J88" s="53"/>
+      <c r="K88" s="53"/>
+      <c r="L88" s="53"/>
+      <c r="M88" s="53"/>
       <c r="N88" s="9"/>
       <c r="O88" s="9"/>
     </row>
@@ -4355,11 +4355,11 @@
       <c r="E89" s="9"/>
       <c r="F89" s="9"/>
       <c r="G89" s="9"/>
-      <c r="H89" s="50" t="s">
+      <c r="H89" s="54" t="s">
         <v>27</v>
       </c>
-      <c r="I89" s="51"/>
-      <c r="J89" s="52"/>
+      <c r="I89" s="55"/>
+      <c r="J89" s="56"/>
       <c r="K89" s="9"/>
       <c r="L89" s="9"/>
       <c r="M89" s="9"/>
@@ -4382,11 +4382,11 @@
         <v>165</v>
       </c>
       <c r="G90" s="48"/>
-      <c r="H90" s="53" t="s">
+      <c r="H90" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="I90" s="53"/>
-      <c r="J90" s="53"/>
+      <c r="I90" s="51"/>
+      <c r="J90" s="51"/>
       <c r="K90" s="9"/>
       <c r="L90" s="9"/>
       <c r="M90" s="9"/>
@@ -4493,20 +4493,20 @@
     </row>
     <row r="95" spans="1:15" ht="15" x14ac:dyDescent="0.25">
       <c r="A95" s="9"/>
-      <c r="B95" s="56" t="s">
+      <c r="B95" s="53" t="s">
         <v>52</v>
       </c>
-      <c r="C95" s="56"/>
-      <c r="D95" s="56"/>
-      <c r="E95" s="56"/>
-      <c r="F95" s="56"/>
-      <c r="G95" s="56"/>
-      <c r="H95" s="56"/>
-      <c r="I95" s="56"/>
-      <c r="J95" s="56"/>
-      <c r="K95" s="56"/>
-      <c r="L95" s="56"/>
-      <c r="M95" s="56"/>
+      <c r="C95" s="53"/>
+      <c r="D95" s="53"/>
+      <c r="E95" s="53"/>
+      <c r="F95" s="53"/>
+      <c r="G95" s="53"/>
+      <c r="H95" s="53"/>
+      <c r="I95" s="53"/>
+      <c r="J95" s="53"/>
+      <c r="K95" s="53"/>
+      <c r="L95" s="53"/>
+      <c r="M95" s="53"/>
       <c r="N95" s="39"/>
       <c r="O95" s="9"/>
     </row>
@@ -4518,11 +4518,11 @@
       <c r="E96" s="39"/>
       <c r="F96" s="9"/>
       <c r="G96" s="9"/>
-      <c r="H96" s="50" t="s">
+      <c r="H96" s="54" t="s">
         <v>27</v>
       </c>
-      <c r="I96" s="51"/>
-      <c r="J96" s="52"/>
+      <c r="I96" s="55"/>
+      <c r="J96" s="56"/>
       <c r="K96" s="9"/>
       <c r="L96" s="9"/>
       <c r="M96" s="9"/>
@@ -4545,11 +4545,11 @@
         <v>173</v>
       </c>
       <c r="G97" s="48"/>
-      <c r="H97" s="53" t="s">
+      <c r="H97" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="I97" s="53"/>
-      <c r="J97" s="53"/>
+      <c r="I97" s="51"/>
+      <c r="J97" s="51"/>
       <c r="K97" s="9"/>
       <c r="L97" s="9"/>
       <c r="M97" s="9"/>
@@ -4605,18 +4605,18 @@
       <c r="B100" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="C100" s="54" t="s">
+      <c r="C100" s="81" t="s">
         <v>56</v>
       </c>
-      <c r="D100" s="55"/>
-      <c r="E100" s="55"/>
-      <c r="F100" s="55"/>
+      <c r="D100" s="60"/>
+      <c r="E100" s="60"/>
+      <c r="F100" s="60"/>
       <c r="G100" s="9"/>
-      <c r="H100" s="50" t="s">
+      <c r="H100" s="54" t="s">
         <v>27</v>
       </c>
-      <c r="I100" s="51"/>
-      <c r="J100" s="52"/>
+      <c r="I100" s="55"/>
+      <c r="J100" s="56"/>
       <c r="K100" s="9"/>
       <c r="L100" s="9"/>
       <c r="M100" s="9"/>
@@ -4633,11 +4633,11 @@
       <c r="G101" s="45" t="s">
         <v>57</v>
       </c>
-      <c r="H101" s="53" t="s">
+      <c r="H101" s="51" t="s">
         <v>14</v>
       </c>
-      <c r="I101" s="53"/>
-      <c r="J101" s="53"/>
+      <c r="I101" s="51"/>
+      <c r="J101" s="51"/>
       <c r="K101" s="9"/>
       <c r="L101" s="9"/>
       <c r="M101" s="9"/>
@@ -4758,13 +4758,13 @@
       <c r="F107" s="5">
         <v>291</v>
       </c>
-      <c r="G107" s="72"/>
-      <c r="H107" s="73"/>
-      <c r="I107" s="73"/>
-      <c r="J107" s="73"/>
-      <c r="K107" s="73"/>
-      <c r="L107" s="73"/>
-      <c r="M107" s="73"/>
+      <c r="G107" s="58"/>
+      <c r="H107" s="59"/>
+      <c r="I107" s="59"/>
+      <c r="J107" s="59"/>
+      <c r="K107" s="59"/>
+      <c r="L107" s="59"/>
+      <c r="M107" s="59"/>
       <c r="N107" s="9"/>
       <c r="O107" s="9"/>
     </row>
@@ -4779,13 +4779,13 @@
       <c r="F108" s="5">
         <v>11</v>
       </c>
-      <c r="G108" s="72"/>
-      <c r="H108" s="73"/>
-      <c r="I108" s="73"/>
-      <c r="J108" s="73"/>
-      <c r="K108" s="73"/>
-      <c r="L108" s="73"/>
-      <c r="M108" s="73"/>
+      <c r="G108" s="58"/>
+      <c r="H108" s="59"/>
+      <c r="I108" s="59"/>
+      <c r="J108" s="59"/>
+      <c r="K108" s="59"/>
+      <c r="L108" s="59"/>
+      <c r="M108" s="59"/>
       <c r="N108" s="9"/>
       <c r="O108" s="9"/>
     </row>
@@ -4811,15 +4811,15 @@
       <c r="D110" s="48"/>
       <c r="E110" s="48"/>
       <c r="F110" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="G110" s="72"/>
-      <c r="H110" s="73"/>
-      <c r="I110" s="73"/>
-      <c r="J110" s="73"/>
-      <c r="K110" s="73"/>
-      <c r="L110" s="73"/>
-      <c r="M110" s="73"/>
+        <v>208</v>
+      </c>
+      <c r="G110" s="58"/>
+      <c r="H110" s="59"/>
+      <c r="I110" s="59"/>
+      <c r="J110" s="59"/>
+      <c r="K110" s="59"/>
+      <c r="L110" s="59"/>
+      <c r="M110" s="59"/>
       <c r="N110" s="39"/>
       <c r="O110" s="9"/>
     </row>
@@ -4869,71 +4869,108 @@
     <sortCondition ref="O5:O52"/>
   </sortState>
   <mergeCells count="191">
-    <mergeCell ref="F67:G67"/>
-    <mergeCell ref="H67:J67"/>
-    <mergeCell ref="F68:G68"/>
-    <mergeCell ref="H68:J68"/>
-    <mergeCell ref="F74:G74"/>
-    <mergeCell ref="H74:J74"/>
-    <mergeCell ref="F75:G75"/>
-    <mergeCell ref="H75:J75"/>
-    <mergeCell ref="F69:G69"/>
-    <mergeCell ref="H69:J69"/>
-    <mergeCell ref="F70:G70"/>
-    <mergeCell ref="H70:J70"/>
-    <mergeCell ref="F71:G71"/>
-    <mergeCell ref="H71:J71"/>
-    <mergeCell ref="F72:G72"/>
-    <mergeCell ref="H72:J72"/>
-    <mergeCell ref="F73:G73"/>
-    <mergeCell ref="H73:J73"/>
-    <mergeCell ref="F62:G62"/>
-    <mergeCell ref="H62:J62"/>
-    <mergeCell ref="F63:G63"/>
-    <mergeCell ref="H63:J63"/>
-    <mergeCell ref="F64:G64"/>
-    <mergeCell ref="H64:J64"/>
-    <mergeCell ref="F65:G65"/>
-    <mergeCell ref="H65:J65"/>
-    <mergeCell ref="F66:G66"/>
-    <mergeCell ref="H66:J66"/>
-    <mergeCell ref="B55:C55"/>
-    <mergeCell ref="I55:K55"/>
-    <mergeCell ref="B56:C56"/>
-    <mergeCell ref="I56:K56"/>
-    <mergeCell ref="B58:M58"/>
-    <mergeCell ref="H59:J59"/>
-    <mergeCell ref="F60:G60"/>
-    <mergeCell ref="H60:J60"/>
-    <mergeCell ref="F61:G61"/>
-    <mergeCell ref="H61:J61"/>
-    <mergeCell ref="B21:D21"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="G21:H21"/>
-    <mergeCell ref="I21:L21"/>
-    <mergeCell ref="B18:D18"/>
-    <mergeCell ref="E18:F18"/>
-    <mergeCell ref="G18:H18"/>
-    <mergeCell ref="I18:L18"/>
-    <mergeCell ref="B19:D19"/>
-    <mergeCell ref="E19:F19"/>
-    <mergeCell ref="G19:H19"/>
-    <mergeCell ref="I19:L19"/>
-    <mergeCell ref="B20:D20"/>
-    <mergeCell ref="E20:F20"/>
-    <mergeCell ref="G20:H20"/>
-    <mergeCell ref="I20:L20"/>
-    <mergeCell ref="I12:L12"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="I13:L13"/>
-    <mergeCell ref="G14:H14"/>
-    <mergeCell ref="I14:L14"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="I15:L15"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="E17:F17"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="I17:L17"/>
+    <mergeCell ref="F91:G91"/>
+    <mergeCell ref="H91:J91"/>
+    <mergeCell ref="F92:G92"/>
+    <mergeCell ref="H92:J92"/>
+    <mergeCell ref="F93:G93"/>
+    <mergeCell ref="H93:J93"/>
+    <mergeCell ref="F85:G85"/>
+    <mergeCell ref="B106:E106"/>
+    <mergeCell ref="B108:E108"/>
+    <mergeCell ref="B107:E107"/>
+    <mergeCell ref="H100:J100"/>
+    <mergeCell ref="H101:J101"/>
+    <mergeCell ref="H102:J102"/>
+    <mergeCell ref="B104:E104"/>
+    <mergeCell ref="C100:F100"/>
+    <mergeCell ref="B95:M95"/>
+    <mergeCell ref="H96:J96"/>
+    <mergeCell ref="F97:G97"/>
+    <mergeCell ref="H97:J97"/>
+    <mergeCell ref="F98:G98"/>
+    <mergeCell ref="H98:J98"/>
+    <mergeCell ref="B105:E105"/>
+    <mergeCell ref="H85:J85"/>
+    <mergeCell ref="F86:G86"/>
+    <mergeCell ref="H86:J86"/>
+    <mergeCell ref="B88:M88"/>
+    <mergeCell ref="H89:J89"/>
+    <mergeCell ref="F90:G90"/>
+    <mergeCell ref="H90:J90"/>
+    <mergeCell ref="F80:G80"/>
+    <mergeCell ref="H80:J80"/>
+    <mergeCell ref="F81:G81"/>
+    <mergeCell ref="H81:J81"/>
+    <mergeCell ref="F82:G82"/>
+    <mergeCell ref="H82:J82"/>
+    <mergeCell ref="F83:G83"/>
+    <mergeCell ref="H83:J83"/>
+    <mergeCell ref="F84:G84"/>
+    <mergeCell ref="H84:J84"/>
+    <mergeCell ref="B43:C43"/>
+    <mergeCell ref="I43:K43"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="I44:K44"/>
+    <mergeCell ref="B77:M77"/>
+    <mergeCell ref="H78:J78"/>
+    <mergeCell ref="F79:G79"/>
+    <mergeCell ref="H79:J79"/>
+    <mergeCell ref="B46:C46"/>
+    <mergeCell ref="B47:C47"/>
+    <mergeCell ref="B48:C48"/>
+    <mergeCell ref="B49:C49"/>
+    <mergeCell ref="B50:C50"/>
+    <mergeCell ref="I46:K46"/>
+    <mergeCell ref="I47:K47"/>
+    <mergeCell ref="I48:K48"/>
+    <mergeCell ref="I49:K49"/>
+    <mergeCell ref="I50:K50"/>
+    <mergeCell ref="B52:C52"/>
+    <mergeCell ref="I52:K52"/>
+    <mergeCell ref="B53:C53"/>
+    <mergeCell ref="I53:K53"/>
+    <mergeCell ref="B54:C54"/>
+    <mergeCell ref="I54:K54"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="I42:K42"/>
+    <mergeCell ref="H24:J24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="B26:C26"/>
+    <mergeCell ref="B27:C27"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="I6:L6"/>
+    <mergeCell ref="I7:L7"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B39:M39"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="I40:K40"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="I41:K41"/>
+    <mergeCell ref="B10:L10"/>
+    <mergeCell ref="B15:D15"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B11:D11"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="G11:H11"/>
+    <mergeCell ref="I11:L11"/>
+    <mergeCell ref="G12:H12"/>
     <mergeCell ref="G107:M107"/>
     <mergeCell ref="B110:E110"/>
     <mergeCell ref="G110:M110"/>
@@ -4958,108 +4995,71 @@
     <mergeCell ref="E6:F6"/>
     <mergeCell ref="G6:H6"/>
     <mergeCell ref="B7:D7"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="I6:L6"/>
-    <mergeCell ref="I7:L7"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B39:M39"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="I40:K40"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="I41:K41"/>
-    <mergeCell ref="B10:L10"/>
-    <mergeCell ref="B15:D15"/>
-    <mergeCell ref="B14:D14"/>
-    <mergeCell ref="B13:D13"/>
-    <mergeCell ref="B12:D12"/>
-    <mergeCell ref="B11:D11"/>
-    <mergeCell ref="E11:F11"/>
-    <mergeCell ref="E12:F12"/>
-    <mergeCell ref="E13:F13"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="I11:L11"/>
-    <mergeCell ref="G12:H12"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="I42:K42"/>
-    <mergeCell ref="H24:J24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="B26:C26"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B34:C34"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B43:C43"/>
-    <mergeCell ref="I43:K43"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="I44:K44"/>
-    <mergeCell ref="B77:M77"/>
-    <mergeCell ref="H78:J78"/>
-    <mergeCell ref="F79:G79"/>
-    <mergeCell ref="H79:J79"/>
-    <mergeCell ref="B46:C46"/>
-    <mergeCell ref="B47:C47"/>
-    <mergeCell ref="B48:C48"/>
-    <mergeCell ref="B49:C49"/>
-    <mergeCell ref="B50:C50"/>
-    <mergeCell ref="I46:K46"/>
-    <mergeCell ref="I47:K47"/>
-    <mergeCell ref="I48:K48"/>
-    <mergeCell ref="I49:K49"/>
-    <mergeCell ref="I50:K50"/>
-    <mergeCell ref="B52:C52"/>
-    <mergeCell ref="I52:K52"/>
-    <mergeCell ref="B53:C53"/>
-    <mergeCell ref="I53:K53"/>
-    <mergeCell ref="B54:C54"/>
-    <mergeCell ref="I54:K54"/>
-    <mergeCell ref="H86:J86"/>
-    <mergeCell ref="B88:M88"/>
-    <mergeCell ref="H89:J89"/>
-    <mergeCell ref="F90:G90"/>
-    <mergeCell ref="H90:J90"/>
-    <mergeCell ref="F80:G80"/>
-    <mergeCell ref="H80:J80"/>
-    <mergeCell ref="F81:G81"/>
-    <mergeCell ref="H81:J81"/>
-    <mergeCell ref="F82:G82"/>
-    <mergeCell ref="H82:J82"/>
-    <mergeCell ref="F83:G83"/>
-    <mergeCell ref="H83:J83"/>
-    <mergeCell ref="F84:G84"/>
-    <mergeCell ref="H84:J84"/>
-    <mergeCell ref="F91:G91"/>
-    <mergeCell ref="H91:J91"/>
-    <mergeCell ref="F92:G92"/>
-    <mergeCell ref="H92:J92"/>
-    <mergeCell ref="F93:G93"/>
-    <mergeCell ref="H93:J93"/>
-    <mergeCell ref="F85:G85"/>
-    <mergeCell ref="B106:E106"/>
-    <mergeCell ref="B108:E108"/>
-    <mergeCell ref="B107:E107"/>
-    <mergeCell ref="H100:J100"/>
-    <mergeCell ref="H101:J101"/>
-    <mergeCell ref="H102:J102"/>
-    <mergeCell ref="B104:E104"/>
-    <mergeCell ref="C100:F100"/>
-    <mergeCell ref="B95:M95"/>
-    <mergeCell ref="H96:J96"/>
-    <mergeCell ref="F97:G97"/>
-    <mergeCell ref="H97:J97"/>
-    <mergeCell ref="F98:G98"/>
-    <mergeCell ref="H98:J98"/>
-    <mergeCell ref="B105:E105"/>
-    <mergeCell ref="H85:J85"/>
-    <mergeCell ref="F86:G86"/>
+    <mergeCell ref="I12:L12"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="I13:L13"/>
+    <mergeCell ref="G14:H14"/>
+    <mergeCell ref="I14:L14"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="I15:L15"/>
+    <mergeCell ref="B17:D17"/>
+    <mergeCell ref="E17:F17"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="I17:L17"/>
+    <mergeCell ref="B21:D21"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="G21:H21"/>
+    <mergeCell ref="I21:L21"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="I18:L18"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="E19:F19"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="I19:L19"/>
+    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="E20:F20"/>
+    <mergeCell ref="G20:H20"/>
+    <mergeCell ref="I20:L20"/>
+    <mergeCell ref="B55:C55"/>
+    <mergeCell ref="I55:K55"/>
+    <mergeCell ref="B56:C56"/>
+    <mergeCell ref="I56:K56"/>
+    <mergeCell ref="B58:M58"/>
+    <mergeCell ref="H59:J59"/>
+    <mergeCell ref="F60:G60"/>
+    <mergeCell ref="H60:J60"/>
+    <mergeCell ref="F61:G61"/>
+    <mergeCell ref="H61:J61"/>
+    <mergeCell ref="F62:G62"/>
+    <mergeCell ref="H62:J62"/>
+    <mergeCell ref="F63:G63"/>
+    <mergeCell ref="H63:J63"/>
+    <mergeCell ref="F64:G64"/>
+    <mergeCell ref="H64:J64"/>
+    <mergeCell ref="F65:G65"/>
+    <mergeCell ref="H65:J65"/>
+    <mergeCell ref="F66:G66"/>
+    <mergeCell ref="H66:J66"/>
+    <mergeCell ref="F67:G67"/>
+    <mergeCell ref="H67:J67"/>
+    <mergeCell ref="F68:G68"/>
+    <mergeCell ref="H68:J68"/>
+    <mergeCell ref="F74:G74"/>
+    <mergeCell ref="H74:J74"/>
+    <mergeCell ref="F75:G75"/>
+    <mergeCell ref="H75:J75"/>
+    <mergeCell ref="F69:G69"/>
+    <mergeCell ref="H69:J69"/>
+    <mergeCell ref="F70:G70"/>
+    <mergeCell ref="H70:J70"/>
+    <mergeCell ref="F71:G71"/>
+    <mergeCell ref="H71:J71"/>
+    <mergeCell ref="F72:G72"/>
+    <mergeCell ref="H72:J72"/>
+    <mergeCell ref="F73:G73"/>
+    <mergeCell ref="H73:J73"/>
   </mergeCells>
   <dataValidations count="4">
     <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D41:D44 F41:F44 H41:H44 L41:L44 D47:D50 F47:F50 H47:H50 L47:L50 D53:D56 F53:F56 H53:H56 L53:L56" xr:uid="{77F1B821-4D03-4E86-9379-0EC9C7C727DB}">

</xml_diff>